<commit_message>
Batch 2 reviewed and applied: out/esES.txt at 49%
Bleu's review: 247 OK, 9 own wording (ranked = "rankeado", "Votar rendirse"). Two lines left open
(SERVER_PERF_LOADED, FRIEND_STATE_IN_GAME) and not applied yet.

Glossary: ranked (rankeado), kick (expulsar), lobby (sala), replay (repetición), leaderboard
(tabla de clasificación), Skill Tier (rango de habilidad) with the tier names.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work/batch2/batch2-review.xlsx
+++ b/work/batch2/batch2-review.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maost\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\[01] Martin\[07] Claude Code\NS2-Spanish-Translation\work\batch2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0CCA24EC-95DB-4637-8840-DFE8321B0BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E7C05FB-FA88-48E7-84D7-48141942E0BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2B8A42E5-E0B3-437F-9640-CBBDC568C62F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{2B8A42E5-E0B3-437F-9640-CBBDC568C62F}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1533" uniqueCount="889">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1798" uniqueCount="900">
   <si>
     <t>Section</t>
   </si>
@@ -2712,6 +2712,39 @@
   </si>
   <si>
     <t>Flagged left</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Use my Spanish</t>
+  </si>
+  <si>
+    <t>Muestra los servidores no rankeados. El nivel de habilidad y experiencia (XP) no son impactados al jugar en servidores no rankeados.</t>
+  </si>
+  <si>
+    <t>OCULTAR NO RANKEADOS</t>
+  </si>
+  <si>
+    <t>RANKEADO</t>
+  </si>
+  <si>
+    <t>¡Este servidor es rankeado! Juega aquí para desbloquear recompensas.</t>
+  </si>
+  <si>
+    <t>Ordena los servidores según sean rankeados o no.</t>
+  </si>
+  <si>
+    <t>NO RANKEADOS</t>
+  </si>
+  <si>
+    <t>¡Este servidor no es rankeado! Aquí no ganarás recompensas.</t>
+  </si>
+  <si>
+    <t>Votar rendirse</t>
+  </si>
+  <si>
+    <t>No se puede iniciar esta votación en una partida competitiva.</t>
   </si>
 </sst>
 </file>
@@ -3272,7 +3305,7 @@
       </c>
       <c r="B10" s="14">
         <f>COUNTA(Review!J2:J258)</f>
-        <v>0</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -3281,7 +3314,7 @@
       </c>
       <c r="B11" s="14">
         <f>ROWS(Review!J2:J258)-COUNTA(Review!J2:J258)</f>
-        <v>257</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -3290,7 +3323,7 @@
       </c>
       <c r="B12" s="14">
         <f>COUNTIFS(Review!G2:G258,"?*",Review!J2:J258,"")</f>
-        <v>46</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3303,21 +3336,21 @@
   <dimension ref="A1:L258"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="26.7109375" customWidth="1"/>
-    <col min="3" max="3" width="44.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="41.140625" customWidth="1"/>
     <col min="4" max="4" width="34.7109375" customWidth="1"/>
     <col min="5" max="5" width="44.7109375" customWidth="1"/>
     <col min="6" max="6" width="8.7109375" customWidth="1"/>
     <col min="7" max="7" width="7.7109375" customWidth="1"/>
     <col min="8" max="8" width="34.7109375" customWidth="1"/>
-    <col min="9" max="9" width="26.7109375" customWidth="1"/>
+    <col min="9" max="9" width="16.140625" customWidth="1"/>
     <col min="10" max="10" width="14.7109375" customWidth="1"/>
     <col min="11" max="11" width="40.7109375" customWidth="1"/>
     <col min="12" max="12" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3377,7 +3410,9 @@
       <c r="G2" s="3"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="5"/>
+      <c r="J2" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K2" s="6"/>
       <c r="L2" s="6"/>
     </row>
@@ -3403,7 +3438,9 @@
       <c r="G3" s="3"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
-      <c r="J3" s="5"/>
+      <c r="J3" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
     </row>
@@ -3427,7 +3464,9 @@
       <c r="G4" s="3"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
-      <c r="J4" s="5"/>
+      <c r="J4" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
     </row>
@@ -3457,7 +3496,9 @@
         <v>28</v>
       </c>
       <c r="I5" s="4"/>
-      <c r="J5" s="5"/>
+      <c r="J5" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
     </row>
@@ -3483,7 +3524,9 @@
       <c r="G6" s="3"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
-      <c r="J6" s="5"/>
+      <c r="J6" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
     </row>
@@ -3507,7 +3550,9 @@
       <c r="G7" s="3"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
-      <c r="J7" s="5"/>
+      <c r="J7" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
     </row>
@@ -3537,7 +3582,9 @@
         <v>39</v>
       </c>
       <c r="I8" s="4"/>
-      <c r="J8" s="5"/>
+      <c r="J8" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
     </row>
@@ -3563,7 +3610,9 @@
       <c r="G9" s="3"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
-      <c r="J9" s="5"/>
+      <c r="J9" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K9" s="6"/>
       <c r="L9" s="6"/>
     </row>
@@ -3589,7 +3638,9 @@
       <c r="G10" s="3"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
-      <c r="J10" s="5"/>
+      <c r="J10" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K10" s="6"/>
       <c r="L10" s="6"/>
     </row>
@@ -3613,7 +3664,9 @@
       <c r="G11" s="3"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
-      <c r="J11" s="5"/>
+      <c r="J11" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K11" s="6"/>
       <c r="L11" s="6"/>
     </row>
@@ -3637,7 +3690,9 @@
       <c r="G12" s="3"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
-      <c r="J12" s="5"/>
+      <c r="J12" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K12" s="6"/>
       <c r="L12" s="6"/>
     </row>
@@ -3661,7 +3716,9 @@
       <c r="G13" s="3"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="5"/>
+      <c r="J13" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K13" s="6"/>
       <c r="L13" s="6"/>
     </row>
@@ -3685,7 +3742,9 @@
       <c r="G14" s="3"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="5"/>
+      <c r="J14" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K14" s="6"/>
       <c r="L14" s="6"/>
     </row>
@@ -3709,7 +3768,9 @@
       <c r="G15" s="3"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
-      <c r="J15" s="5"/>
+      <c r="J15" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K15" s="6"/>
       <c r="L15" s="6"/>
     </row>
@@ -3735,7 +3796,9 @@
         <v>62</v>
       </c>
       <c r="I16" s="4"/>
-      <c r="J16" s="5"/>
+      <c r="J16" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K16" s="6"/>
       <c r="L16" s="6"/>
     </row>
@@ -3763,7 +3826,9 @@
         <v>65</v>
       </c>
       <c r="I17" s="4"/>
-      <c r="J17" s="5"/>
+      <c r="J17" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
     </row>
@@ -3795,7 +3860,9 @@
       <c r="I18" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="J18" s="5"/>
+      <c r="J18" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K18" s="6"/>
       <c r="L18" s="6"/>
     </row>
@@ -3821,7 +3888,9 @@
       <c r="G19" s="3"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-      <c r="J19" s="5"/>
+      <c r="J19" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K19" s="6"/>
       <c r="L19" s="6"/>
     </row>
@@ -3847,7 +3916,9 @@
       <c r="G20" s="3"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
-      <c r="J20" s="5"/>
+      <c r="J20" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K20" s="6"/>
       <c r="L20" s="6"/>
     </row>
@@ -3873,7 +3944,9 @@
       <c r="G21" s="3"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="5"/>
+      <c r="J21" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K21" s="6"/>
       <c r="L21" s="6"/>
     </row>
@@ -3901,7 +3974,9 @@
         <v>82</v>
       </c>
       <c r="I22" s="4"/>
-      <c r="J22" s="5"/>
+      <c r="J22" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K22" s="6"/>
       <c r="L22" s="6"/>
     </row>
@@ -3927,7 +4002,9 @@
       <c r="G23" s="3"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
-      <c r="J23" s="5"/>
+      <c r="J23" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K23" s="6"/>
       <c r="L23" s="6"/>
     </row>
@@ -3953,7 +4030,9 @@
       <c r="G24" s="3"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
-      <c r="J24" s="5"/>
+      <c r="J24" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K24" s="6"/>
       <c r="L24" s="6"/>
     </row>
@@ -3979,7 +4058,9 @@
       <c r="G25" s="3"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
-      <c r="J25" s="5"/>
+      <c r="J25" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K25" s="6"/>
       <c r="L25" s="6"/>
     </row>
@@ -4005,7 +4086,9 @@
       <c r="G26" s="3"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
-      <c r="J26" s="5"/>
+      <c r="J26" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K26" s="6"/>
       <c r="L26" s="6"/>
     </row>
@@ -4031,7 +4114,9 @@
       <c r="G27" s="3"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
-      <c r="J27" s="5"/>
+      <c r="J27" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K27" s="6"/>
       <c r="L27" s="6"/>
     </row>
@@ -4055,7 +4140,9 @@
       <c r="G28" s="3"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
-      <c r="J28" s="5"/>
+      <c r="J28" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K28" s="6"/>
       <c r="L28" s="6"/>
     </row>
@@ -4081,7 +4168,9 @@
       <c r="G29" s="3"/>
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
-      <c r="J29" s="5"/>
+      <c r="J29" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K29" s="6"/>
       <c r="L29" s="6"/>
     </row>
@@ -4107,7 +4196,9 @@
       <c r="G30" s="3"/>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
-      <c r="J30" s="5"/>
+      <c r="J30" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K30" s="6"/>
       <c r="L30" s="6"/>
     </row>
@@ -4133,7 +4224,9 @@
       <c r="G31" s="3"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
-      <c r="J31" s="5"/>
+      <c r="J31" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K31" s="6"/>
       <c r="L31" s="6"/>
     </row>
@@ -4159,7 +4252,9 @@
       <c r="G32" s="3"/>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
-      <c r="J32" s="5"/>
+      <c r="J32" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K32" s="6"/>
       <c r="L32" s="6"/>
     </row>
@@ -4185,7 +4280,9 @@
       <c r="G33" s="3"/>
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
-      <c r="J33" s="5"/>
+      <c r="J33" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K33" s="6"/>
       <c r="L33" s="6"/>
     </row>
@@ -4209,7 +4306,9 @@
       <c r="G34" s="3"/>
       <c r="H34" s="4"/>
       <c r="I34" s="4"/>
-      <c r="J34" s="5"/>
+      <c r="J34" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K34" s="6"/>
       <c r="L34" s="6"/>
     </row>
@@ -4233,7 +4332,9 @@
       <c r="G35" s="3"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
-      <c r="J35" s="5"/>
+      <c r="J35" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K35" s="6"/>
       <c r="L35" s="6"/>
     </row>
@@ -4257,7 +4358,9 @@
       <c r="G36" s="3"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
-      <c r="J36" s="5"/>
+      <c r="J36" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K36" s="6"/>
       <c r="L36" s="6"/>
     </row>
@@ -4283,7 +4386,9 @@
         <v>127</v>
       </c>
       <c r="I37" s="4"/>
-      <c r="J37" s="5"/>
+      <c r="J37" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K37" s="6"/>
       <c r="L37" s="6"/>
     </row>
@@ -4307,7 +4412,9 @@
       <c r="G38" s="3"/>
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
-      <c r="J38" s="5"/>
+      <c r="J38" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K38" s="6"/>
       <c r="L38" s="6"/>
     </row>
@@ -4331,7 +4438,9 @@
       <c r="G39" s="3"/>
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
-      <c r="J39" s="5"/>
+      <c r="J39" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K39" s="6"/>
       <c r="L39" s="6"/>
     </row>
@@ -4355,7 +4464,9 @@
       <c r="G40" s="3"/>
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
-      <c r="J40" s="5"/>
+      <c r="J40" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K40" s="6"/>
       <c r="L40" s="6"/>
     </row>
@@ -4379,7 +4490,9 @@
       <c r="G41" s="3"/>
       <c r="H41" s="4"/>
       <c r="I41" s="4"/>
-      <c r="J41" s="5"/>
+      <c r="J41" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K41" s="6"/>
       <c r="L41" s="6"/>
     </row>
@@ -4405,7 +4518,9 @@
       <c r="G42" s="3"/>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
-      <c r="J42" s="5"/>
+      <c r="J42" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K42" s="6"/>
       <c r="L42" s="6"/>
     </row>
@@ -4429,7 +4544,9 @@
       <c r="G43" s="3"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
-      <c r="J43" s="5"/>
+      <c r="J43" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K43" s="6"/>
       <c r="L43" s="6"/>
     </row>
@@ -4455,7 +4572,9 @@
       <c r="G44" s="3"/>
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
-      <c r="J44" s="5"/>
+      <c r="J44" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K44" s="6"/>
       <c r="L44" s="6"/>
     </row>
@@ -4481,7 +4600,9 @@
       <c r="G45" s="3"/>
       <c r="H45" s="4"/>
       <c r="I45" s="4"/>
-      <c r="J45" s="5"/>
+      <c r="J45" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K45" s="6"/>
       <c r="L45" s="6"/>
     </row>
@@ -4505,7 +4626,9 @@
       <c r="G46" s="3"/>
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
-      <c r="J46" s="5"/>
+      <c r="J46" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K46" s="6"/>
       <c r="L46" s="6"/>
     </row>
@@ -4529,7 +4652,9 @@
       <c r="G47" s="3"/>
       <c r="H47" s="4"/>
       <c r="I47" s="4"/>
-      <c r="J47" s="5"/>
+      <c r="J47" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K47" s="6"/>
       <c r="L47" s="6"/>
     </row>
@@ -4553,7 +4678,9 @@
       <c r="G48" s="3"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4"/>
-      <c r="J48" s="5"/>
+      <c r="J48" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K48" s="6"/>
       <c r="L48" s="6"/>
     </row>
@@ -4577,7 +4704,9 @@
       <c r="G49" s="3"/>
       <c r="H49" s="4"/>
       <c r="I49" s="4"/>
-      <c r="J49" s="5"/>
+      <c r="J49" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K49" s="6"/>
       <c r="L49" s="6"/>
     </row>
@@ -4607,7 +4736,9 @@
         <v>167</v>
       </c>
       <c r="I50" s="4"/>
-      <c r="J50" s="5"/>
+      <c r="J50" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K50" s="6"/>
       <c r="L50" s="6"/>
     </row>
@@ -4633,7 +4764,9 @@
       <c r="G51" s="3"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4"/>
-      <c r="J51" s="5"/>
+      <c r="J51" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K51" s="6"/>
       <c r="L51" s="6"/>
     </row>
@@ -4657,7 +4790,9 @@
       <c r="G52" s="3"/>
       <c r="H52" s="4"/>
       <c r="I52" s="4"/>
-      <c r="J52" s="5"/>
+      <c r="J52" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K52" s="6"/>
       <c r="L52" s="6"/>
     </row>
@@ -4681,7 +4816,9 @@
       <c r="G53" s="3"/>
       <c r="H53" s="4"/>
       <c r="I53" s="4"/>
-      <c r="J53" s="5"/>
+      <c r="J53" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K53" s="6"/>
       <c r="L53" s="6"/>
     </row>
@@ -4705,7 +4842,9 @@
       <c r="G54" s="3"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
-      <c r="J54" s="5"/>
+      <c r="J54" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K54" s="6"/>
       <c r="L54" s="6"/>
     </row>
@@ -4735,8 +4874,12 @@
         <v>184</v>
       </c>
       <c r="I55" s="4"/>
-      <c r="J55" s="5"/>
-      <c r="K55" s="6"/>
+      <c r="J55" s="5" t="s">
+        <v>890</v>
+      </c>
+      <c r="K55" s="6" t="s">
+        <v>891</v>
+      </c>
       <c r="L55" s="6"/>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.2">
@@ -4759,7 +4902,9 @@
       <c r="G56" s="3"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4"/>
-      <c r="J56" s="5"/>
+      <c r="J56" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K56" s="6"/>
       <c r="L56" s="6"/>
     </row>
@@ -4783,7 +4928,9 @@
       <c r="G57" s="3"/>
       <c r="H57" s="4"/>
       <c r="I57" s="4"/>
-      <c r="J57" s="5"/>
+      <c r="J57" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K57" s="6"/>
       <c r="L57" s="6"/>
     </row>
@@ -4809,7 +4956,9 @@
       <c r="G58" s="3"/>
       <c r="H58" s="4"/>
       <c r="I58" s="4"/>
-      <c r="J58" s="5"/>
+      <c r="J58" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K58" s="6"/>
       <c r="L58" s="6"/>
     </row>
@@ -4833,7 +4982,9 @@
       <c r="G59" s="3"/>
       <c r="H59" s="4"/>
       <c r="I59" s="4"/>
-      <c r="J59" s="5"/>
+      <c r="J59" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K59" s="6"/>
       <c r="L59" s="6"/>
     </row>
@@ -4859,7 +5010,9 @@
       <c r="I60" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="J60" s="5"/>
+      <c r="J60" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K60" s="6"/>
       <c r="L60" s="6"/>
     </row>
@@ -4889,7 +5042,9 @@
         <v>205</v>
       </c>
       <c r="I61" s="4"/>
-      <c r="J61" s="5"/>
+      <c r="J61" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K61" s="6"/>
       <c r="L61" s="6"/>
     </row>
@@ -4915,7 +5070,9 @@
       <c r="G62" s="3"/>
       <c r="H62" s="4"/>
       <c r="I62" s="4"/>
-      <c r="J62" s="5"/>
+      <c r="J62" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K62" s="6"/>
       <c r="L62" s="6"/>
     </row>
@@ -4941,7 +5098,9 @@
       <c r="G63" s="3"/>
       <c r="H63" s="4"/>
       <c r="I63" s="4"/>
-      <c r="J63" s="5"/>
+      <c r="J63" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K63" s="6"/>
       <c r="L63" s="6"/>
     </row>
@@ -4965,7 +5124,9 @@
       <c r="G64" s="3"/>
       <c r="H64" s="4"/>
       <c r="I64" s="4"/>
-      <c r="J64" s="5"/>
+      <c r="J64" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K64" s="6"/>
       <c r="L64" s="6"/>
     </row>
@@ -4991,7 +5152,9 @@
       <c r="G65" s="3"/>
       <c r="H65" s="4"/>
       <c r="I65" s="4"/>
-      <c r="J65" s="5"/>
+      <c r="J65" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K65" s="6"/>
       <c r="L65" s="6"/>
     </row>
@@ -5015,7 +5178,9 @@
       <c r="G66" s="3"/>
       <c r="H66" s="4"/>
       <c r="I66" s="4"/>
-      <c r="J66" s="5"/>
+      <c r="J66" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K66" s="6"/>
       <c r="L66" s="6"/>
     </row>
@@ -5041,7 +5206,9 @@
       <c r="G67" s="3"/>
       <c r="H67" s="4"/>
       <c r="I67" s="4"/>
-      <c r="J67" s="5"/>
+      <c r="J67" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K67" s="6"/>
       <c r="L67" s="6"/>
     </row>
@@ -5065,7 +5232,9 @@
       <c r="G68" s="3"/>
       <c r="H68" s="4"/>
       <c r="I68" s="4"/>
-      <c r="J68" s="5"/>
+      <c r="J68" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K68" s="6"/>
       <c r="L68" s="6"/>
     </row>
@@ -5089,7 +5258,9 @@
       <c r="G69" s="3"/>
       <c r="H69" s="4"/>
       <c r="I69" s="4"/>
-      <c r="J69" s="5"/>
+      <c r="J69" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K69" s="6"/>
       <c r="L69" s="6"/>
     </row>
@@ -5113,7 +5284,9 @@
       <c r="G70" s="3"/>
       <c r="H70" s="4"/>
       <c r="I70" s="4"/>
-      <c r="J70" s="5"/>
+      <c r="J70" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K70" s="6"/>
       <c r="L70" s="6"/>
     </row>
@@ -5137,7 +5310,9 @@
       <c r="G71" s="3"/>
       <c r="H71" s="4"/>
       <c r="I71" s="4"/>
-      <c r="J71" s="5"/>
+      <c r="J71" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K71" s="6"/>
       <c r="L71" s="6"/>
     </row>
@@ -5161,7 +5336,9 @@
       <c r="G72" s="3"/>
       <c r="H72" s="4"/>
       <c r="I72" s="4"/>
-      <c r="J72" s="5"/>
+      <c r="J72" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K72" s="6"/>
       <c r="L72" s="6"/>
     </row>
@@ -5187,7 +5364,9 @@
       <c r="G73" s="3"/>
       <c r="H73" s="4"/>
       <c r="I73" s="4"/>
-      <c r="J73" s="5"/>
+      <c r="J73" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K73" s="6"/>
       <c r="L73" s="6"/>
     </row>
@@ -5213,7 +5392,9 @@
       <c r="G74" s="3"/>
       <c r="H74" s="4"/>
       <c r="I74" s="4"/>
-      <c r="J74" s="5"/>
+      <c r="J74" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K74" s="6"/>
       <c r="L74" s="6"/>
     </row>
@@ -5237,7 +5418,9 @@
       <c r="G75" s="3"/>
       <c r="H75" s="4"/>
       <c r="I75" s="4"/>
-      <c r="J75" s="5"/>
+      <c r="J75" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K75" s="6"/>
       <c r="L75" s="6"/>
     </row>
@@ -5261,7 +5444,9 @@
       <c r="G76" s="3"/>
       <c r="H76" s="4"/>
       <c r="I76" s="4"/>
-      <c r="J76" s="5"/>
+      <c r="J76" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K76" s="6"/>
       <c r="L76" s="6"/>
     </row>
@@ -5285,7 +5470,9 @@
       <c r="G77" s="3"/>
       <c r="H77" s="4"/>
       <c r="I77" s="4"/>
-      <c r="J77" s="5"/>
+      <c r="J77" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K77" s="6"/>
       <c r="L77" s="6"/>
     </row>
@@ -5309,7 +5496,9 @@
       <c r="G78" s="3"/>
       <c r="H78" s="4"/>
       <c r="I78" s="4"/>
-      <c r="J78" s="5"/>
+      <c r="J78" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K78" s="6"/>
       <c r="L78" s="6"/>
     </row>
@@ -5333,7 +5522,9 @@
       <c r="G79" s="3"/>
       <c r="H79" s="4"/>
       <c r="I79" s="4"/>
-      <c r="J79" s="5"/>
+      <c r="J79" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K79" s="6"/>
       <c r="L79" s="6"/>
     </row>
@@ -5359,7 +5550,9 @@
       <c r="G80" s="3"/>
       <c r="H80" s="4"/>
       <c r="I80" s="4"/>
-      <c r="J80" s="5"/>
+      <c r="J80" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K80" s="6"/>
       <c r="L80" s="6"/>
     </row>
@@ -5383,7 +5576,9 @@
       <c r="G81" s="3"/>
       <c r="H81" s="4"/>
       <c r="I81" s="4"/>
-      <c r="J81" s="5"/>
+      <c r="J81" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K81" s="6"/>
       <c r="L81" s="6"/>
     </row>
@@ -5409,7 +5604,9 @@
       <c r="G82" s="3"/>
       <c r="H82" s="4"/>
       <c r="I82" s="4"/>
-      <c r="J82" s="5"/>
+      <c r="J82" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K82" s="6"/>
       <c r="L82" s="6"/>
     </row>
@@ -5433,7 +5630,9 @@
       <c r="G83" s="3"/>
       <c r="H83" s="4"/>
       <c r="I83" s="4"/>
-      <c r="J83" s="5"/>
+      <c r="J83" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K83" s="6"/>
       <c r="L83" s="6"/>
     </row>
@@ -5465,8 +5664,12 @@
       <c r="I84" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="J84" s="5"/>
-      <c r="K84" s="6"/>
+      <c r="J84" s="5" t="s">
+        <v>890</v>
+      </c>
+      <c r="K84" s="6" t="s">
+        <v>892</v>
+      </c>
       <c r="L84" s="6"/>
     </row>
     <row r="85" spans="1:12" ht="25.5" x14ac:dyDescent="0.2">
@@ -5491,7 +5694,9 @@
         <v>277</v>
       </c>
       <c r="I85" s="4"/>
-      <c r="J85" s="5"/>
+      <c r="J85" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K85" s="6"/>
       <c r="L85" s="6"/>
     </row>
@@ -5519,8 +5724,12 @@
         <v>282</v>
       </c>
       <c r="I86" s="4"/>
-      <c r="J86" s="5"/>
-      <c r="K86" s="6"/>
+      <c r="J86" s="5" t="s">
+        <v>890</v>
+      </c>
+      <c r="K86" s="6" t="s">
+        <v>893</v>
+      </c>
       <c r="L86" s="6"/>
     </row>
     <row r="87" spans="1:12" ht="38.25" x14ac:dyDescent="0.2">
@@ -5549,8 +5758,12 @@
         <v>287</v>
       </c>
       <c r="I87" s="4"/>
-      <c r="J87" s="5"/>
-      <c r="K87" s="6"/>
+      <c r="J87" s="5" t="s">
+        <v>890</v>
+      </c>
+      <c r="K87" s="6" t="s">
+        <v>894</v>
+      </c>
       <c r="L87" s="6"/>
     </row>
     <row r="88" spans="1:12" ht="25.5" x14ac:dyDescent="0.2">
@@ -5579,8 +5792,12 @@
         <v>292</v>
       </c>
       <c r="I88" s="4"/>
-      <c r="J88" s="5"/>
-      <c r="K88" s="6"/>
+      <c r="J88" s="5" t="s">
+        <v>890</v>
+      </c>
+      <c r="K88" s="6" t="s">
+        <v>895</v>
+      </c>
       <c r="L88" s="6"/>
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.2">
@@ -5603,7 +5820,9 @@
       <c r="G89" s="3"/>
       <c r="H89" s="4"/>
       <c r="I89" s="4"/>
-      <c r="J89" s="5"/>
+      <c r="J89" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K89" s="6"/>
       <c r="L89" s="6"/>
     </row>
@@ -5631,7 +5850,9 @@
       <c r="I90" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="J90" s="5"/>
+      <c r="J90" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K90" s="6"/>
       <c r="L90" s="6"/>
     </row>
@@ -5655,7 +5876,9 @@
       <c r="G91" s="3"/>
       <c r="H91" s="4"/>
       <c r="I91" s="4"/>
-      <c r="J91" s="5"/>
+      <c r="J91" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K91" s="6"/>
       <c r="L91" s="6"/>
     </row>
@@ -5679,7 +5902,9 @@
       <c r="G92" s="3"/>
       <c r="H92" s="4"/>
       <c r="I92" s="4"/>
-      <c r="J92" s="5"/>
+      <c r="J92" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K92" s="6"/>
       <c r="L92" s="6"/>
     </row>
@@ -5709,7 +5934,9 @@
         <v>311</v>
       </c>
       <c r="I93" s="4"/>
-      <c r="J93" s="5"/>
+      <c r="J93" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K93" s="6"/>
       <c r="L93" s="6"/>
     </row>
@@ -5735,7 +5962,9 @@
       <c r="G94" s="3"/>
       <c r="H94" s="4"/>
       <c r="I94" s="4"/>
-      <c r="J94" s="5"/>
+      <c r="J94" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K94" s="6"/>
       <c r="L94" s="6"/>
     </row>
@@ -5765,7 +5994,9 @@
         <v>319</v>
       </c>
       <c r="I95" s="4"/>
-      <c r="J95" s="5"/>
+      <c r="J95" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K95" s="6"/>
       <c r="L95" s="6"/>
     </row>
@@ -5789,7 +6020,9 @@
       <c r="G96" s="3"/>
       <c r="H96" s="4"/>
       <c r="I96" s="4"/>
-      <c r="J96" s="5"/>
+      <c r="J96" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K96" s="6"/>
       <c r="L96" s="6"/>
     </row>
@@ -5815,7 +6048,9 @@
       <c r="G97" s="3"/>
       <c r="H97" s="4"/>
       <c r="I97" s="4"/>
-      <c r="J97" s="5"/>
+      <c r="J97" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K97" s="6"/>
       <c r="L97" s="6"/>
     </row>
@@ -5841,7 +6076,9 @@
       <c r="G98" s="3"/>
       <c r="H98" s="4"/>
       <c r="I98" s="4"/>
-      <c r="J98" s="5"/>
+      <c r="J98" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K98" s="6"/>
       <c r="L98" s="6"/>
     </row>
@@ -5867,7 +6104,9 @@
       <c r="G99" s="3"/>
       <c r="H99" s="4"/>
       <c r="I99" s="4"/>
-      <c r="J99" s="5"/>
+      <c r="J99" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K99" s="6"/>
       <c r="L99" s="6"/>
     </row>
@@ -5891,7 +6130,9 @@
       <c r="G100" s="3"/>
       <c r="H100" s="4"/>
       <c r="I100" s="4"/>
-      <c r="J100" s="5"/>
+      <c r="J100" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K100" s="6"/>
       <c r="L100" s="6"/>
     </row>
@@ -5915,7 +6156,9 @@
       <c r="G101" s="3"/>
       <c r="H101" s="4"/>
       <c r="I101" s="4"/>
-      <c r="J101" s="5"/>
+      <c r="J101" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K101" s="6"/>
       <c r="L101" s="6"/>
     </row>
@@ -5941,7 +6184,9 @@
       <c r="G102" s="3"/>
       <c r="H102" s="4"/>
       <c r="I102" s="4"/>
-      <c r="J102" s="5"/>
+      <c r="J102" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K102" s="6"/>
       <c r="L102" s="6"/>
     </row>
@@ -5965,7 +6210,9 @@
       <c r="G103" s="3"/>
       <c r="H103" s="4"/>
       <c r="I103" s="4"/>
-      <c r="J103" s="5"/>
+      <c r="J103" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K103" s="6"/>
       <c r="L103" s="6"/>
     </row>
@@ -5991,7 +6238,9 @@
         <v>346</v>
       </c>
       <c r="I104" s="4"/>
-      <c r="J104" s="5"/>
+      <c r="J104" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K104" s="6"/>
       <c r="L104" s="6"/>
     </row>
@@ -6015,7 +6264,9 @@
       <c r="G105" s="3"/>
       <c r="H105" s="4"/>
       <c r="I105" s="4"/>
-      <c r="J105" s="5"/>
+      <c r="J105" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K105" s="6"/>
       <c r="L105" s="6"/>
     </row>
@@ -6039,7 +6290,9 @@
       <c r="G106" s="3"/>
       <c r="H106" s="4"/>
       <c r="I106" s="4"/>
-      <c r="J106" s="5"/>
+      <c r="J106" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K106" s="6"/>
       <c r="L106" s="6"/>
     </row>
@@ -6069,7 +6322,9 @@
         <v>357</v>
       </c>
       <c r="I107" s="4"/>
-      <c r="J107" s="5"/>
+      <c r="J107" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K107" s="6"/>
       <c r="L107" s="6"/>
     </row>
@@ -6093,7 +6348,9 @@
       <c r="G108" s="3"/>
       <c r="H108" s="4"/>
       <c r="I108" s="4"/>
-      <c r="J108" s="5"/>
+      <c r="J108" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K108" s="6"/>
       <c r="L108" s="6"/>
     </row>
@@ -6123,7 +6380,9 @@
         <v>365</v>
       </c>
       <c r="I109" s="4"/>
-      <c r="J109" s="5"/>
+      <c r="J109" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K109" s="6"/>
       <c r="L109" s="6"/>
     </row>
@@ -6147,7 +6406,9 @@
       <c r="G110" s="3"/>
       <c r="H110" s="4"/>
       <c r="I110" s="4"/>
-      <c r="J110" s="5"/>
+      <c r="J110" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K110" s="6"/>
       <c r="L110" s="6"/>
     </row>
@@ -6177,8 +6438,12 @@
       <c r="I111" s="10" t="s">
         <v>373</v>
       </c>
-      <c r="J111" s="5"/>
-      <c r="K111" s="6"/>
+      <c r="J111" s="5" t="s">
+        <v>890</v>
+      </c>
+      <c r="K111" s="6" t="s">
+        <v>896</v>
+      </c>
       <c r="L111" s="6"/>
     </row>
     <row r="112" spans="1:12" ht="38.25" x14ac:dyDescent="0.2">
@@ -6205,7 +6470,9 @@
         <v>377</v>
       </c>
       <c r="I112" s="4"/>
-      <c r="J112" s="5"/>
+      <c r="J112" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K112" s="6"/>
       <c r="L112" s="6"/>
     </row>
@@ -6229,7 +6496,9 @@
       <c r="G113" s="3"/>
       <c r="H113" s="4"/>
       <c r="I113" s="4"/>
-      <c r="J113" s="5"/>
+      <c r="J113" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K113" s="6"/>
       <c r="L113" s="6"/>
     </row>
@@ -6255,7 +6524,9 @@
       <c r="G114" s="3"/>
       <c r="H114" s="4"/>
       <c r="I114" s="4"/>
-      <c r="J114" s="5"/>
+      <c r="J114" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K114" s="6"/>
       <c r="L114" s="6"/>
     </row>
@@ -6285,8 +6556,12 @@
         <v>292</v>
       </c>
       <c r="I115" s="4"/>
-      <c r="J115" s="5"/>
-      <c r="K115" s="6"/>
+      <c r="J115" s="5" t="s">
+        <v>890</v>
+      </c>
+      <c r="K115" s="6" t="s">
+        <v>897</v>
+      </c>
       <c r="L115" s="6"/>
     </row>
     <row r="116" spans="1:12" ht="25.5" x14ac:dyDescent="0.2">
@@ -6309,7 +6584,9 @@
       <c r="G116" s="3"/>
       <c r="H116" s="4"/>
       <c r="I116" s="4"/>
-      <c r="J116" s="5"/>
+      <c r="J116" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K116" s="6"/>
       <c r="L116" s="6"/>
     </row>
@@ -6333,7 +6610,9 @@
       <c r="G117" s="3"/>
       <c r="H117" s="4"/>
       <c r="I117" s="4"/>
-      <c r="J117" s="5"/>
+      <c r="J117" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K117" s="6"/>
       <c r="L117" s="6"/>
     </row>
@@ -6359,7 +6638,9 @@
       <c r="G118" s="3"/>
       <c r="H118" s="4"/>
       <c r="I118" s="4"/>
-      <c r="J118" s="5"/>
+      <c r="J118" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K118" s="6"/>
       <c r="L118" s="6"/>
     </row>
@@ -6383,7 +6664,9 @@
       <c r="G119" s="3"/>
       <c r="H119" s="4"/>
       <c r="I119" s="4"/>
-      <c r="J119" s="5"/>
+      <c r="J119" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K119" s="6"/>
       <c r="L119" s="6"/>
     </row>
@@ -6409,7 +6692,9 @@
       <c r="G120" s="3"/>
       <c r="H120" s="4"/>
       <c r="I120" s="4"/>
-      <c r="J120" s="5"/>
+      <c r="J120" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K120" s="6"/>
       <c r="L120" s="6"/>
     </row>
@@ -6435,7 +6720,9 @@
       <c r="G121" s="3"/>
       <c r="H121" s="4"/>
       <c r="I121" s="4"/>
-      <c r="J121" s="5"/>
+      <c r="J121" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K121" s="6"/>
       <c r="L121" s="6"/>
     </row>
@@ -6463,7 +6750,9 @@
         <v>409</v>
       </c>
       <c r="I122" s="4"/>
-      <c r="J122" s="5"/>
+      <c r="J122" s="5" t="s">
+        <v>890</v>
+      </c>
       <c r="K122" s="6"/>
       <c r="L122" s="6"/>
     </row>
@@ -6493,7 +6782,9 @@
         <v>413</v>
       </c>
       <c r="I123" s="4"/>
-      <c r="J123" s="5"/>
+      <c r="J123" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K123" s="6"/>
       <c r="L123" s="6"/>
     </row>
@@ -6519,7 +6810,9 @@
       <c r="G124" s="3"/>
       <c r="H124" s="4"/>
       <c r="I124" s="4"/>
-      <c r="J124" s="5"/>
+      <c r="J124" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K124" s="6"/>
       <c r="L124" s="6"/>
     </row>
@@ -6543,7 +6836,9 @@
       <c r="G125" s="3"/>
       <c r="H125" s="4"/>
       <c r="I125" s="4"/>
-      <c r="J125" s="5"/>
+      <c r="J125" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K125" s="6"/>
       <c r="L125" s="6"/>
     </row>
@@ -6567,7 +6862,9 @@
       <c r="G126" s="3"/>
       <c r="H126" s="4"/>
       <c r="I126" s="4"/>
-      <c r="J126" s="5"/>
+      <c r="J126" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K126" s="6"/>
       <c r="L126" s="6"/>
     </row>
@@ -6593,7 +6890,9 @@
         <v>427</v>
       </c>
       <c r="I127" s="4"/>
-      <c r="J127" s="5"/>
+      <c r="J127" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K127" s="6"/>
       <c r="L127" s="6"/>
     </row>
@@ -6617,7 +6916,9 @@
       <c r="G128" s="3"/>
       <c r="H128" s="4"/>
       <c r="I128" s="4"/>
-      <c r="J128" s="5"/>
+      <c r="J128" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K128" s="6"/>
       <c r="L128" s="6"/>
     </row>
@@ -6643,7 +6944,9 @@
       <c r="G129" s="3"/>
       <c r="H129" s="4"/>
       <c r="I129" s="4"/>
-      <c r="J129" s="5"/>
+      <c r="J129" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K129" s="6"/>
       <c r="L129" s="6"/>
     </row>
@@ -6667,7 +6970,9 @@
       <c r="G130" s="3"/>
       <c r="H130" s="4"/>
       <c r="I130" s="4"/>
-      <c r="J130" s="5"/>
+      <c r="J130" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K130" s="6"/>
       <c r="L130" s="6"/>
     </row>
@@ -6691,7 +6996,9 @@
       <c r="G131" s="3"/>
       <c r="H131" s="4"/>
       <c r="I131" s="4"/>
-      <c r="J131" s="5"/>
+      <c r="J131" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K131" s="6"/>
       <c r="L131" s="6"/>
     </row>
@@ -6715,7 +7022,9 @@
       <c r="G132" s="3"/>
       <c r="H132" s="4"/>
       <c r="I132" s="4"/>
-      <c r="J132" s="5"/>
+      <c r="J132" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K132" s="6"/>
       <c r="L132" s="6"/>
     </row>
@@ -6739,7 +7048,9 @@
       <c r="G133" s="3"/>
       <c r="H133" s="4"/>
       <c r="I133" s="4"/>
-      <c r="J133" s="5"/>
+      <c r="J133" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K133" s="6"/>
       <c r="L133" s="6"/>
     </row>
@@ -6763,7 +7074,9 @@
       <c r="G134" s="3"/>
       <c r="H134" s="4"/>
       <c r="I134" s="4"/>
-      <c r="J134" s="5"/>
+      <c r="J134" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K134" s="6"/>
       <c r="L134" s="6"/>
     </row>
@@ -6787,7 +7100,9 @@
       <c r="G135" s="3"/>
       <c r="H135" s="4"/>
       <c r="I135" s="4"/>
-      <c r="J135" s="5"/>
+      <c r="J135" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K135" s="6"/>
       <c r="L135" s="6"/>
     </row>
@@ -6813,7 +7128,9 @@
       <c r="G136" s="3"/>
       <c r="H136" s="4"/>
       <c r="I136" s="4"/>
-      <c r="J136" s="5"/>
+      <c r="J136" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K136" s="6"/>
       <c r="L136" s="6"/>
     </row>
@@ -6839,7 +7156,9 @@
         <v>457</v>
       </c>
       <c r="I137" s="4"/>
-      <c r="J137" s="5"/>
+      <c r="J137" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K137" s="6"/>
       <c r="L137" s="6"/>
     </row>
@@ -6863,7 +7182,9 @@
       <c r="G138" s="3"/>
       <c r="H138" s="4"/>
       <c r="I138" s="4"/>
-      <c r="J138" s="5"/>
+      <c r="J138" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K138" s="6"/>
       <c r="L138" s="6"/>
     </row>
@@ -6887,7 +7208,9 @@
       <c r="G139" s="3"/>
       <c r="H139" s="4"/>
       <c r="I139" s="4"/>
-      <c r="J139" s="5"/>
+      <c r="J139" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K139" s="6"/>
       <c r="L139" s="6"/>
     </row>
@@ -6911,7 +7234,9 @@
       <c r="G140" s="3"/>
       <c r="H140" s="4"/>
       <c r="I140" s="4"/>
-      <c r="J140" s="5"/>
+      <c r="J140" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K140" s="6"/>
       <c r="L140" s="6"/>
     </row>
@@ -6935,7 +7260,9 @@
       <c r="G141" s="3"/>
       <c r="H141" s="4"/>
       <c r="I141" s="4"/>
-      <c r="J141" s="5"/>
+      <c r="J141" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K141" s="6"/>
       <c r="L141" s="6"/>
     </row>
@@ -6959,7 +7286,9 @@
       <c r="G142" s="3"/>
       <c r="H142" s="4"/>
       <c r="I142" s="4"/>
-      <c r="J142" s="5"/>
+      <c r="J142" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K142" s="6"/>
       <c r="L142" s="6"/>
     </row>
@@ -6983,7 +7312,9 @@
       <c r="G143" s="3"/>
       <c r="H143" s="4"/>
       <c r="I143" s="4"/>
-      <c r="J143" s="5"/>
+      <c r="J143" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K143" s="6"/>
       <c r="L143" s="6"/>
     </row>
@@ -7031,7 +7362,9 @@
       <c r="G145" s="3"/>
       <c r="H145" s="4"/>
       <c r="I145" s="4"/>
-      <c r="J145" s="5"/>
+      <c r="J145" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K145" s="6"/>
       <c r="L145" s="6"/>
     </row>
@@ -7055,7 +7388,9 @@
       <c r="G146" s="3"/>
       <c r="H146" s="4"/>
       <c r="I146" s="4"/>
-      <c r="J146" s="5"/>
+      <c r="J146" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K146" s="6"/>
       <c r="L146" s="6"/>
     </row>
@@ -7079,7 +7414,9 @@
       <c r="G147" s="3"/>
       <c r="H147" s="4"/>
       <c r="I147" s="4"/>
-      <c r="J147" s="5"/>
+      <c r="J147" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K147" s="6"/>
       <c r="L147" s="6"/>
     </row>
@@ -7103,7 +7440,9 @@
       <c r="G148" s="3"/>
       <c r="H148" s="4"/>
       <c r="I148" s="4"/>
-      <c r="J148" s="5"/>
+      <c r="J148" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K148" s="6"/>
       <c r="L148" s="6"/>
     </row>
@@ -7127,7 +7466,9 @@
       <c r="G149" s="3"/>
       <c r="H149" s="4"/>
       <c r="I149" s="4"/>
-      <c r="J149" s="5"/>
+      <c r="J149" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K149" s="6"/>
       <c r="L149" s="6"/>
     </row>
@@ -7151,7 +7492,9 @@
       <c r="G150" s="3"/>
       <c r="H150" s="4"/>
       <c r="I150" s="4"/>
-      <c r="J150" s="5"/>
+      <c r="J150" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K150" s="6"/>
       <c r="L150" s="6"/>
     </row>
@@ -7179,7 +7522,9 @@
         <v>500</v>
       </c>
       <c r="I151" s="4"/>
-      <c r="J151" s="5"/>
+      <c r="J151" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K151" s="6"/>
       <c r="L151" s="6"/>
     </row>
@@ -7203,7 +7548,9 @@
       <c r="G152" s="3"/>
       <c r="H152" s="4"/>
       <c r="I152" s="4"/>
-      <c r="J152" s="5"/>
+      <c r="J152" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K152" s="6"/>
       <c r="L152" s="6"/>
     </row>
@@ -7227,7 +7574,9 @@
       <c r="G153" s="3"/>
       <c r="H153" s="4"/>
       <c r="I153" s="4"/>
-      <c r="J153" s="5"/>
+      <c r="J153" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K153" s="6"/>
       <c r="L153" s="6"/>
     </row>
@@ -7251,7 +7600,9 @@
       <c r="G154" s="3"/>
       <c r="H154" s="4"/>
       <c r="I154" s="4"/>
-      <c r="J154" s="5"/>
+      <c r="J154" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K154" s="6"/>
       <c r="L154" s="6"/>
     </row>
@@ -7275,7 +7626,9 @@
       <c r="G155" s="3"/>
       <c r="H155" s="4"/>
       <c r="I155" s="4"/>
-      <c r="J155" s="5"/>
+      <c r="J155" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K155" s="6"/>
       <c r="L155" s="6"/>
     </row>
@@ -7299,7 +7652,9 @@
       <c r="G156" s="3"/>
       <c r="H156" s="4"/>
       <c r="I156" s="4"/>
-      <c r="J156" s="5"/>
+      <c r="J156" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K156" s="6"/>
       <c r="L156" s="6"/>
     </row>
@@ -7323,7 +7678,9 @@
       <c r="G157" s="3"/>
       <c r="H157" s="4"/>
       <c r="I157" s="4"/>
-      <c r="J157" s="5"/>
+      <c r="J157" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K157" s="6"/>
       <c r="L157" s="6"/>
     </row>
@@ -7347,7 +7704,9 @@
       <c r="G158" s="3"/>
       <c r="H158" s="4"/>
       <c r="I158" s="4"/>
-      <c r="J158" s="5"/>
+      <c r="J158" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K158" s="6"/>
       <c r="L158" s="6"/>
     </row>
@@ -7371,7 +7730,9 @@
       <c r="G159" s="3"/>
       <c r="H159" s="4"/>
       <c r="I159" s="4"/>
-      <c r="J159" s="5"/>
+      <c r="J159" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K159" s="6"/>
       <c r="L159" s="6"/>
     </row>
@@ -7397,7 +7758,9 @@
       <c r="G160" s="3"/>
       <c r="H160" s="4"/>
       <c r="I160" s="4"/>
-      <c r="J160" s="5"/>
+      <c r="J160" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K160" s="6"/>
       <c r="L160" s="6"/>
     </row>
@@ -7421,7 +7784,9 @@
       <c r="G161" s="3"/>
       <c r="H161" s="4"/>
       <c r="I161" s="4"/>
-      <c r="J161" s="5"/>
+      <c r="J161" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K161" s="6"/>
       <c r="L161" s="6"/>
     </row>
@@ -7445,7 +7810,9 @@
       <c r="G162" s="3"/>
       <c r="H162" s="4"/>
       <c r="I162" s="4"/>
-      <c r="J162" s="5"/>
+      <c r="J162" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K162" s="6"/>
       <c r="L162" s="6"/>
     </row>
@@ -7469,7 +7836,9 @@
       <c r="G163" s="3"/>
       <c r="H163" s="4"/>
       <c r="I163" s="4"/>
-      <c r="J163" s="5"/>
+      <c r="J163" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K163" s="6"/>
       <c r="L163" s="6"/>
     </row>
@@ -7493,7 +7862,9 @@
       <c r="G164" s="3"/>
       <c r="H164" s="4"/>
       <c r="I164" s="4"/>
-      <c r="J164" s="5"/>
+      <c r="J164" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K164" s="6"/>
       <c r="L164" s="6"/>
     </row>
@@ -7517,7 +7888,9 @@
       <c r="G165" s="3"/>
       <c r="H165" s="4"/>
       <c r="I165" s="4"/>
-      <c r="J165" s="5"/>
+      <c r="J165" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K165" s="6"/>
       <c r="L165" s="6"/>
     </row>
@@ -7541,7 +7914,9 @@
       <c r="G166" s="3"/>
       <c r="H166" s="4"/>
       <c r="I166" s="4"/>
-      <c r="J166" s="5"/>
+      <c r="J166" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K166" s="6"/>
       <c r="L166" s="6"/>
     </row>
@@ -7565,7 +7940,9 @@
       <c r="G167" s="3"/>
       <c r="H167" s="4"/>
       <c r="I167" s="4"/>
-      <c r="J167" s="5"/>
+      <c r="J167" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K167" s="6"/>
       <c r="L167" s="6"/>
     </row>
@@ -7589,7 +7966,9 @@
       <c r="G168" s="3"/>
       <c r="H168" s="4"/>
       <c r="I168" s="4"/>
-      <c r="J168" s="5"/>
+      <c r="J168" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K168" s="6"/>
       <c r="L168" s="6"/>
     </row>
@@ -7615,7 +7994,9 @@
         <v>554</v>
       </c>
       <c r="I169" s="4"/>
-      <c r="J169" s="5"/>
+      <c r="J169" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K169" s="6"/>
       <c r="L169" s="6"/>
     </row>
@@ -7639,7 +8020,9 @@
       <c r="G170" s="3"/>
       <c r="H170" s="4"/>
       <c r="I170" s="4"/>
-      <c r="J170" s="5"/>
+      <c r="J170" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K170" s="6"/>
       <c r="L170" s="6"/>
     </row>
@@ -7665,7 +8048,9 @@
         <v>561</v>
       </c>
       <c r="I171" s="4"/>
-      <c r="J171" s="5"/>
+      <c r="J171" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K171" s="6"/>
       <c r="L171" s="6"/>
     </row>
@@ -7689,7 +8074,9 @@
       <c r="G172" s="3"/>
       <c r="H172" s="4"/>
       <c r="I172" s="4"/>
-      <c r="J172" s="5"/>
+      <c r="J172" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K172" s="6"/>
       <c r="L172" s="6"/>
     </row>
@@ -7713,7 +8100,9 @@
       <c r="G173" s="3"/>
       <c r="H173" s="4"/>
       <c r="I173" s="4"/>
-      <c r="J173" s="5"/>
+      <c r="J173" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K173" s="6"/>
       <c r="L173" s="6"/>
     </row>
@@ -7737,7 +8126,9 @@
       <c r="G174" s="3"/>
       <c r="H174" s="4"/>
       <c r="I174" s="4"/>
-      <c r="J174" s="5"/>
+      <c r="J174" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K174" s="6"/>
       <c r="L174" s="6"/>
     </row>
@@ -7761,7 +8152,9 @@
       <c r="G175" s="3"/>
       <c r="H175" s="4"/>
       <c r="I175" s="4"/>
-      <c r="J175" s="5"/>
+      <c r="J175" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K175" s="6"/>
       <c r="L175" s="6"/>
     </row>
@@ -7785,7 +8178,9 @@
       <c r="G176" s="3"/>
       <c r="H176" s="4"/>
       <c r="I176" s="4"/>
-      <c r="J176" s="5"/>
+      <c r="J176" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K176" s="6"/>
       <c r="L176" s="6"/>
     </row>
@@ -7809,7 +8204,9 @@
       <c r="G177" s="3"/>
       <c r="H177" s="4"/>
       <c r="I177" s="4"/>
-      <c r="J177" s="5"/>
+      <c r="J177" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K177" s="6"/>
       <c r="L177" s="6"/>
     </row>
@@ -7835,7 +8232,9 @@
       <c r="G178" s="3"/>
       <c r="H178" s="4"/>
       <c r="I178" s="4"/>
-      <c r="J178" s="5"/>
+      <c r="J178" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K178" s="6"/>
       <c r="L178" s="6"/>
     </row>
@@ -7865,7 +8264,9 @@
         <v>587</v>
       </c>
       <c r="I179" s="4"/>
-      <c r="J179" s="5"/>
+      <c r="J179" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K179" s="6"/>
       <c r="L179" s="6"/>
     </row>
@@ -7891,7 +8292,9 @@
       <c r="I180" s="10" t="s">
         <v>591</v>
       </c>
-      <c r="J180" s="5"/>
+      <c r="J180" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K180" s="6"/>
       <c r="L180" s="6"/>
     </row>
@@ -7917,7 +8320,9 @@
       <c r="G181" s="3"/>
       <c r="H181" s="4"/>
       <c r="I181" s="4"/>
-      <c r="J181" s="5"/>
+      <c r="J181" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K181" s="6"/>
       <c r="L181" s="6"/>
     </row>
@@ -7943,7 +8348,9 @@
       <c r="G182" s="3"/>
       <c r="H182" s="4"/>
       <c r="I182" s="4"/>
-      <c r="J182" s="5"/>
+      <c r="J182" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K182" s="6"/>
       <c r="L182" s="6"/>
     </row>
@@ -7973,7 +8380,9 @@
         <v>602</v>
       </c>
       <c r="I183" s="4"/>
-      <c r="J183" s="5"/>
+      <c r="J183" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K183" s="6"/>
       <c r="L183" s="6"/>
     </row>
@@ -8003,7 +8412,9 @@
         <v>607</v>
       </c>
       <c r="I184" s="4"/>
-      <c r="J184" s="5"/>
+      <c r="J184" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K184" s="6"/>
       <c r="L184" s="6"/>
     </row>
@@ -8033,7 +8444,9 @@
         <v>612</v>
       </c>
       <c r="I185" s="4"/>
-      <c r="J185" s="5"/>
+      <c r="J185" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K185" s="6"/>
       <c r="L185" s="6"/>
     </row>
@@ -8059,7 +8472,9 @@
       <c r="G186" s="3"/>
       <c r="H186" s="4"/>
       <c r="I186" s="4"/>
-      <c r="J186" s="5"/>
+      <c r="J186" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K186" s="6"/>
       <c r="L186" s="6"/>
     </row>
@@ -8085,7 +8500,9 @@
         <v>619</v>
       </c>
       <c r="I187" s="4"/>
-      <c r="J187" s="5"/>
+      <c r="J187" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K187" s="6"/>
       <c r="L187" s="6"/>
     </row>
@@ -8115,7 +8532,9 @@
         <v>624</v>
       </c>
       <c r="I188" s="4"/>
-      <c r="J188" s="5"/>
+      <c r="J188" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K188" s="6"/>
       <c r="L188" s="6"/>
     </row>
@@ -8139,7 +8558,9 @@
       <c r="G189" s="3"/>
       <c r="H189" s="4"/>
       <c r="I189" s="4"/>
-      <c r="J189" s="5"/>
+      <c r="J189" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K189" s="6"/>
       <c r="L189" s="6"/>
     </row>
@@ -8169,7 +8590,9 @@
         <v>632</v>
       </c>
       <c r="I190" s="4"/>
-      <c r="J190" s="5"/>
+      <c r="J190" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K190" s="6"/>
       <c r="L190" s="6"/>
     </row>
@@ -8195,7 +8618,9 @@
       <c r="G191" s="3"/>
       <c r="H191" s="4"/>
       <c r="I191" s="4"/>
-      <c r="J191" s="5"/>
+      <c r="J191" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K191" s="6"/>
       <c r="L191" s="6"/>
     </row>
@@ -8225,7 +8650,9 @@
         <v>640</v>
       </c>
       <c r="I192" s="4"/>
-      <c r="J192" s="5"/>
+      <c r="J192" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K192" s="6"/>
       <c r="L192" s="6"/>
     </row>
@@ -8255,7 +8682,9 @@
         <v>645</v>
       </c>
       <c r="I193" s="4"/>
-      <c r="J193" s="5"/>
+      <c r="J193" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K193" s="6"/>
       <c r="L193" s="6"/>
     </row>
@@ -8285,7 +8714,9 @@
         <v>650</v>
       </c>
       <c r="I194" s="4"/>
-      <c r="J194" s="5"/>
+      <c r="J194" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K194" s="6"/>
       <c r="L194" s="6"/>
     </row>
@@ -8311,7 +8742,9 @@
       <c r="G195" s="3"/>
       <c r="H195" s="4"/>
       <c r="I195" s="4"/>
-      <c r="J195" s="5"/>
+      <c r="J195" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K195" s="6"/>
       <c r="L195" s="6"/>
     </row>
@@ -8337,7 +8770,9 @@
       <c r="G196" s="3"/>
       <c r="H196" s="4"/>
       <c r="I196" s="4"/>
-      <c r="J196" s="5"/>
+      <c r="J196" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K196" s="6"/>
       <c r="L196" s="6"/>
     </row>
@@ -8363,7 +8798,9 @@
       <c r="G197" s="3"/>
       <c r="H197" s="4"/>
       <c r="I197" s="4"/>
-      <c r="J197" s="5"/>
+      <c r="J197" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K197" s="6"/>
       <c r="L197" s="6"/>
     </row>
@@ -8389,7 +8826,9 @@
       <c r="G198" s="3"/>
       <c r="H198" s="4"/>
       <c r="I198" s="4"/>
-      <c r="J198" s="5"/>
+      <c r="J198" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K198" s="6"/>
       <c r="L198" s="6"/>
     </row>
@@ -8419,7 +8858,9 @@
         <v>667</v>
       </c>
       <c r="I199" s="4"/>
-      <c r="J199" s="5"/>
+      <c r="J199" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K199" s="6"/>
       <c r="L199" s="6"/>
     </row>
@@ -8449,7 +8890,9 @@
         <v>672</v>
       </c>
       <c r="I200" s="4"/>
-      <c r="J200" s="5"/>
+      <c r="J200" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K200" s="6"/>
       <c r="L200" s="6"/>
     </row>
@@ -8479,7 +8922,9 @@
         <v>677</v>
       </c>
       <c r="I201" s="4"/>
-      <c r="J201" s="5"/>
+      <c r="J201" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K201" s="6"/>
       <c r="L201" s="6"/>
     </row>
@@ -8507,7 +8952,9 @@
         <v>682</v>
       </c>
       <c r="I202" s="4"/>
-      <c r="J202" s="5"/>
+      <c r="J202" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K202" s="6"/>
       <c r="L202" s="6"/>
     </row>
@@ -8531,7 +8978,9 @@
       <c r="G203" s="3"/>
       <c r="H203" s="4"/>
       <c r="I203" s="4"/>
-      <c r="J203" s="5"/>
+      <c r="J203" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K203" s="6"/>
       <c r="L203" s="6"/>
     </row>
@@ -8555,7 +9004,9 @@
       <c r="G204" s="3"/>
       <c r="H204" s="4"/>
       <c r="I204" s="4"/>
-      <c r="J204" s="5"/>
+      <c r="J204" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K204" s="6"/>
       <c r="L204" s="6"/>
     </row>
@@ -8579,7 +9030,9 @@
       <c r="G205" s="3"/>
       <c r="H205" s="4"/>
       <c r="I205" s="4"/>
-      <c r="J205" s="5"/>
+      <c r="J205" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K205" s="6"/>
       <c r="L205" s="6"/>
     </row>
@@ -8603,7 +9056,9 @@
       <c r="G206" s="3"/>
       <c r="H206" s="4"/>
       <c r="I206" s="4"/>
-      <c r="J206" s="5"/>
+      <c r="J206" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K206" s="6"/>
       <c r="L206" s="6"/>
     </row>
@@ -8627,7 +9082,9 @@
       <c r="G207" s="3"/>
       <c r="H207" s="4"/>
       <c r="I207" s="4"/>
-      <c r="J207" s="5"/>
+      <c r="J207" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K207" s="6"/>
       <c r="L207" s="6"/>
     </row>
@@ -8653,7 +9110,9 @@
       <c r="G208" s="3"/>
       <c r="H208" s="4"/>
       <c r="I208" s="4"/>
-      <c r="J208" s="5"/>
+      <c r="J208" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K208" s="6"/>
       <c r="L208" s="6"/>
     </row>
@@ -8679,7 +9138,9 @@
       <c r="G209" s="3"/>
       <c r="H209" s="4"/>
       <c r="I209" s="4"/>
-      <c r="J209" s="5"/>
+      <c r="J209" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K209" s="6"/>
       <c r="L209" s="6"/>
     </row>
@@ -8705,8 +9166,12 @@
       <c r="G210" s="3"/>
       <c r="H210" s="4"/>
       <c r="I210" s="4"/>
-      <c r="J210" s="5"/>
-      <c r="K210" s="6"/>
+      <c r="J210" s="5" t="s">
+        <v>890</v>
+      </c>
+      <c r="K210" s="6" t="s">
+        <v>898</v>
+      </c>
       <c r="L210" s="6"/>
     </row>
     <row r="211" spans="1:12" ht="38.25" x14ac:dyDescent="0.2">
@@ -8735,7 +9200,9 @@
         <v>713</v>
       </c>
       <c r="I211" s="4"/>
-      <c r="J211" s="5"/>
+      <c r="J211" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K211" s="6"/>
       <c r="L211" s="6"/>
     </row>
@@ -8761,7 +9228,9 @@
       <c r="G212" s="3"/>
       <c r="H212" s="4"/>
       <c r="I212" s="4"/>
-      <c r="J212" s="5"/>
+      <c r="J212" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K212" s="6"/>
       <c r="L212" s="6"/>
     </row>
@@ -8791,7 +9260,9 @@
         <v>722</v>
       </c>
       <c r="I213" s="4"/>
-      <c r="J213" s="5"/>
+      <c r="J213" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K213" s="6"/>
       <c r="L213" s="6"/>
     </row>
@@ -8815,7 +9286,9 @@
       <c r="G214" s="3"/>
       <c r="H214" s="4"/>
       <c r="I214" s="4"/>
-      <c r="J214" s="5"/>
+      <c r="J214" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K214" s="6"/>
       <c r="L214" s="6"/>
     </row>
@@ -8841,7 +9314,9 @@
       <c r="G215" s="3"/>
       <c r="H215" s="4"/>
       <c r="I215" s="4"/>
-      <c r="J215" s="5"/>
+      <c r="J215" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K215" s="6"/>
       <c r="L215" s="6"/>
     </row>
@@ -8865,7 +9340,9 @@
       <c r="G216" s="3"/>
       <c r="H216" s="4"/>
       <c r="I216" s="4"/>
-      <c r="J216" s="5"/>
+      <c r="J216" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K216" s="6"/>
       <c r="L216" s="6"/>
     </row>
@@ -8889,7 +9366,9 @@
       <c r="G217" s="3"/>
       <c r="H217" s="4"/>
       <c r="I217" s="4"/>
-      <c r="J217" s="5"/>
+      <c r="J217" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K217" s="6"/>
       <c r="L217" s="6"/>
     </row>
@@ -8915,7 +9394,9 @@
       <c r="G218" s="3"/>
       <c r="H218" s="4"/>
       <c r="I218" s="4"/>
-      <c r="J218" s="5"/>
+      <c r="J218" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K218" s="6"/>
       <c r="L218" s="6"/>
     </row>
@@ -8939,7 +9420,9 @@
       <c r="G219" s="3"/>
       <c r="H219" s="4"/>
       <c r="I219" s="4"/>
-      <c r="J219" s="5"/>
+      <c r="J219" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K219" s="6"/>
       <c r="L219" s="6"/>
     </row>
@@ -8965,7 +9448,9 @@
       <c r="G220" s="3"/>
       <c r="H220" s="4"/>
       <c r="I220" s="4"/>
-      <c r="J220" s="5"/>
+      <c r="J220" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K220" s="6"/>
       <c r="L220" s="6"/>
     </row>
@@ -8995,7 +9480,9 @@
         <v>750</v>
       </c>
       <c r="I221" s="4"/>
-      <c r="J221" s="5"/>
+      <c r="J221" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K221" s="6"/>
       <c r="L221" s="6"/>
     </row>
@@ -9025,7 +9512,9 @@
         <v>755</v>
       </c>
       <c r="I222" s="4"/>
-      <c r="J222" s="5"/>
+      <c r="J222" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K222" s="6"/>
       <c r="L222" s="6"/>
     </row>
@@ -9049,7 +9538,9 @@
       <c r="G223" s="3"/>
       <c r="H223" s="4"/>
       <c r="I223" s="4"/>
-      <c r="J223" s="5"/>
+      <c r="J223" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K223" s="6"/>
       <c r="L223" s="6"/>
     </row>
@@ -9075,7 +9566,9 @@
       <c r="G224" s="3"/>
       <c r="H224" s="4"/>
       <c r="I224" s="4"/>
-      <c r="J224" s="5"/>
+      <c r="J224" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K224" s="6"/>
       <c r="L224" s="6"/>
     </row>
@@ -9101,7 +9594,9 @@
       <c r="G225" s="3"/>
       <c r="H225" s="4"/>
       <c r="I225" s="4"/>
-      <c r="J225" s="5"/>
+      <c r="J225" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K225" s="6"/>
       <c r="L225" s="6"/>
     </row>
@@ -9125,7 +9620,9 @@
       <c r="G226" s="3"/>
       <c r="H226" s="4"/>
       <c r="I226" s="4"/>
-      <c r="J226" s="5"/>
+      <c r="J226" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K226" s="6"/>
       <c r="L226" s="6"/>
     </row>
@@ -9149,7 +9646,9 @@
       <c r="G227" s="3"/>
       <c r="H227" s="4"/>
       <c r="I227" s="4"/>
-      <c r="J227" s="5"/>
+      <c r="J227" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K227" s="6"/>
       <c r="L227" s="6"/>
     </row>
@@ -9173,7 +9672,9 @@
       <c r="G228" s="3"/>
       <c r="H228" s="4"/>
       <c r="I228" s="4"/>
-      <c r="J228" s="5"/>
+      <c r="J228" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K228" s="6"/>
       <c r="L228" s="6"/>
     </row>
@@ -9199,7 +9700,9 @@
       <c r="G229" s="3"/>
       <c r="H229" s="4"/>
       <c r="I229" s="4"/>
-      <c r="J229" s="5"/>
+      <c r="J229" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K229" s="6"/>
       <c r="L229" s="6"/>
     </row>
@@ -9227,7 +9730,9 @@
         <v>782</v>
       </c>
       <c r="I230" s="4"/>
-      <c r="J230" s="5"/>
+      <c r="J230" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K230" s="6"/>
       <c r="L230" s="6"/>
     </row>
@@ -9253,7 +9758,9 @@
       <c r="G231" s="3"/>
       <c r="H231" s="4"/>
       <c r="I231" s="4"/>
-      <c r="J231" s="5"/>
+      <c r="J231" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K231" s="6"/>
       <c r="L231" s="6"/>
     </row>
@@ -9281,7 +9788,9 @@
       <c r="I232" s="10" t="s">
         <v>790</v>
       </c>
-      <c r="J232" s="5"/>
+      <c r="J232" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K232" s="6"/>
       <c r="L232" s="6"/>
     </row>
@@ -9311,7 +9820,9 @@
         <v>795</v>
       </c>
       <c r="I233" s="4"/>
-      <c r="J233" s="5"/>
+      <c r="J233" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K233" s="6"/>
       <c r="L233" s="6"/>
     </row>
@@ -9335,7 +9846,9 @@
       <c r="G234" s="3"/>
       <c r="H234" s="4"/>
       <c r="I234" s="4"/>
-      <c r="J234" s="5"/>
+      <c r="J234" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K234" s="6"/>
       <c r="L234" s="6"/>
     </row>
@@ -9361,7 +9874,9 @@
       <c r="G235" s="3"/>
       <c r="H235" s="4"/>
       <c r="I235" s="4"/>
-      <c r="J235" s="5"/>
+      <c r="J235" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K235" s="6"/>
       <c r="L235" s="6"/>
     </row>
@@ -9387,7 +9902,9 @@
       <c r="G236" s="3"/>
       <c r="H236" s="4"/>
       <c r="I236" s="4"/>
-      <c r="J236" s="5"/>
+      <c r="J236" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K236" s="6"/>
       <c r="L236" s="6"/>
     </row>
@@ -9413,7 +9930,9 @@
       <c r="G237" s="3"/>
       <c r="H237" s="4"/>
       <c r="I237" s="4"/>
-      <c r="J237" s="5"/>
+      <c r="J237" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K237" s="6"/>
       <c r="L237" s="6"/>
     </row>
@@ -9441,8 +9960,12 @@
         <v>813</v>
       </c>
       <c r="I238" s="4"/>
-      <c r="J238" s="5"/>
-      <c r="K238" s="6"/>
+      <c r="J238" s="5" t="s">
+        <v>889</v>
+      </c>
+      <c r="K238" s="6" t="s">
+        <v>899</v>
+      </c>
       <c r="L238" s="6"/>
     </row>
     <row r="239" spans="1:12" ht="25.5" x14ac:dyDescent="0.2">
@@ -9467,7 +9990,9 @@
       <c r="I239" s="10" t="s">
         <v>790</v>
       </c>
-      <c r="J239" s="5"/>
+      <c r="J239" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K239" s="6"/>
       <c r="L239" s="6"/>
     </row>
@@ -9491,7 +10016,9 @@
       <c r="G240" s="3"/>
       <c r="H240" s="4"/>
       <c r="I240" s="4"/>
-      <c r="J240" s="5"/>
+      <c r="J240" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K240" s="6"/>
       <c r="L240" s="6"/>
     </row>
@@ -9515,7 +10042,9 @@
       <c r="G241" s="3"/>
       <c r="H241" s="4"/>
       <c r="I241" s="4"/>
-      <c r="J241" s="5"/>
+      <c r="J241" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K241" s="6"/>
       <c r="L241" s="6"/>
     </row>
@@ -9539,7 +10068,9 @@
       <c r="G242" s="3"/>
       <c r="H242" s="4"/>
       <c r="I242" s="4"/>
-      <c r="J242" s="5"/>
+      <c r="J242" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K242" s="6"/>
       <c r="L242" s="6"/>
     </row>
@@ -9563,7 +10094,9 @@
       <c r="G243" s="3"/>
       <c r="H243" s="4"/>
       <c r="I243" s="4"/>
-      <c r="J243" s="5"/>
+      <c r="J243" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K243" s="6"/>
       <c r="L243" s="6"/>
     </row>
@@ -9589,7 +10122,9 @@
       <c r="I244" s="10" t="s">
         <v>831</v>
       </c>
-      <c r="J244" s="5"/>
+      <c r="J244" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K244" s="6"/>
       <c r="L244" s="6"/>
     </row>
@@ -9613,7 +10148,9 @@
       <c r="G245" s="3"/>
       <c r="H245" s="4"/>
       <c r="I245" s="4"/>
-      <c r="J245" s="5"/>
+      <c r="J245" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K245" s="6"/>
       <c r="L245" s="6"/>
     </row>
@@ -9637,7 +10174,9 @@
       <c r="G246" s="3"/>
       <c r="H246" s="4"/>
       <c r="I246" s="4"/>
-      <c r="J246" s="5"/>
+      <c r="J246" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K246" s="6"/>
       <c r="L246" s="6"/>
     </row>
@@ -9661,7 +10200,9 @@
       <c r="G247" s="3"/>
       <c r="H247" s="4"/>
       <c r="I247" s="4"/>
-      <c r="J247" s="5"/>
+      <c r="J247" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K247" s="6"/>
       <c r="L247" s="6"/>
     </row>
@@ -9685,7 +10226,9 @@
       <c r="G248" s="3"/>
       <c r="H248" s="4"/>
       <c r="I248" s="4"/>
-      <c r="J248" s="5"/>
+      <c r="J248" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K248" s="6"/>
       <c r="L248" s="6"/>
     </row>
@@ -9713,7 +10256,9 @@
         <v>846</v>
       </c>
       <c r="I249" s="4"/>
-      <c r="J249" s="5"/>
+      <c r="J249" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K249" s="6"/>
       <c r="L249" s="6"/>
     </row>
@@ -9741,7 +10286,9 @@
         <v>849</v>
       </c>
       <c r="I250" s="4"/>
-      <c r="J250" s="5"/>
+      <c r="J250" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K250" s="6"/>
       <c r="L250" s="6"/>
     </row>
@@ -9769,7 +10316,9 @@
         <v>853</v>
       </c>
       <c r="I251" s="4"/>
-      <c r="J251" s="5"/>
+      <c r="J251" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K251" s="6"/>
       <c r="L251" s="6"/>
     </row>
@@ -9797,7 +10346,9 @@
         <v>857</v>
       </c>
       <c r="I252" s="4"/>
-      <c r="J252" s="5"/>
+      <c r="J252" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K252" s="6"/>
       <c r="L252" s="6"/>
     </row>
@@ -9825,7 +10376,9 @@
         <v>861</v>
       </c>
       <c r="I253" s="4"/>
-      <c r="J253" s="5"/>
+      <c r="J253" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K253" s="6"/>
       <c r="L253" s="6"/>
     </row>
@@ -9855,7 +10408,9 @@
       <c r="I254" s="10" t="s">
         <v>790</v>
       </c>
-      <c r="J254" s="5"/>
+      <c r="J254" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K254" s="6"/>
       <c r="L254" s="6"/>
     </row>
@@ -9883,7 +10438,9 @@
         <v>853</v>
       </c>
       <c r="I255" s="4"/>
-      <c r="J255" s="5"/>
+      <c r="J255" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K255" s="6"/>
       <c r="L255" s="6"/>
     </row>
@@ -9909,7 +10466,9 @@
         <v>871</v>
       </c>
       <c r="I256" s="4"/>
-      <c r="J256" s="5"/>
+      <c r="J256" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K256" s="6"/>
       <c r="L256" s="6"/>
     </row>
@@ -9937,7 +10496,9 @@
         <v>853</v>
       </c>
       <c r="I257" s="4"/>
-      <c r="J257" s="5"/>
+      <c r="J257" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K257" s="6"/>
       <c r="L257" s="6"/>
     </row>
@@ -9961,7 +10522,9 @@
       <c r="G258" s="3"/>
       <c r="H258" s="4"/>
       <c r="I258" s="4"/>
-      <c r="J258" s="5"/>
+      <c r="J258" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="K258" s="6"/>
       <c r="L258" s="6"/>
     </row>

</xml_diff>